<commit_message>
Add supervisor proposal, fix Koskidex size figure
Add Magistrale/Tesi/proposta-relatore.md: a two-page pitch for prof.
Bonnici, to hand over after the first Algoritmi per l'IA lecture on
21 September 2026. It frames the work as building the missing yardstick
rather than as having written a search engine, states the three ranking
defects with file and line, and commits up front to writing relevance
judgments by hand before observing the engine's answers.

Correct the size of Koskidex everywhere it appeared. The 130k figure came
from the GitHub languages API, which reports BYTES, not lines. The repo is
2,853 lines of Go plus 2,063 of tests. Fixed in appunti.md and in both
copies of the selection spreadsheet.
</commit_message>
<xml_diff>
--- a/Magistrale/Tesi/selezione-progetti.xlsx
+++ b/Magistrale/Tesi/selezione-progetti.xlsx
@@ -555,7 +555,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A33"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
   </cols>
@@ -775,7 +775,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>Traccia gia' aperta e unico candidato con codice interamente proprio. L'ingegneria c'e' (circa 130k righe di Go); manca la parte scientifica: valutazione su collezioni standard (BEIR, MS MARCO), curve recall@k contro latenza, confronto con Meilisearch, Tantivy ed Elasticsearch e soprattutto uno studio sulla fusione lessicale piu' densa (RRF contro pesatura), che e' il candidato piu' forte a diventare la domanda di tesi.</t>
+          <t>Traccia gia' aperta e unico candidato con codice interamente proprio. L'ingegneria c'e' (2.850 righe di codice piu' 2.060 di test); manca la parte scientifica: valutazione su collezioni standard (BEIR, MS MARCO), curve recall@k contro latenza, confronto con Meilisearch, Tantivy ed Elasticsearch e soprattutto uno studio sulla fusione lessicale piu' densa (RRF contro pesatura), che e' il candidato piu' forte a diventare la domanda di tesi.</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2080,7 +2080,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
@@ -2726,7 +2726,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M383"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
@@ -3186,7 +3186,7 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>Traccia gia' aperta e unico candidato con codice interamente proprio. L'ingegneria c'e' (circa 130k righe di Go); manca la parte scientifica: valutazione su collezioni standard (BEIR, MS MARCO), curve recall@k contro latenza, confronto con Meilisearch, Tantivy ed Elasticsearch e soprattutto uno studio sulla fusione lessicale piu' densa (RRF contro pesatura), che e' il candidato piu' forte a diventare la domanda di tesi.</t>
+          <t>Traccia gia' aperta e unico candidato con codice interamente proprio. L'ingegneria c'e' (2.850 righe di codice piu' 2.060 di test); manca la parte scientifica: valutazione su collezioni standard (BEIR, MS MARCO), curve recall@k contro latenza, confronto con Meilisearch, Tantivy ed Elasticsearch e soprattutto uno studio sulla fusione lessicale piu' densa (RRF contro pesatura), che e' il candidato piu' forte a diventare la domanda di tesi.</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">

</xml_diff>